<commit_message>
Add demo assistance contacts and referral data
</commit_message>
<xml_diff>
--- a/assets/data/kedah-silver-data-blueprint.xlsx
+++ b/assets/data/kedah-silver-data-blueprint.xlsx
@@ -52,7 +52,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
         <fgColor rgb="00F3F6F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00123B31"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -87,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -97,6 +102,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -469,27 +477,27 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>How to use</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Privacy rule</t>
         </is>
@@ -534,7 +542,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -544,42 +552,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>weight_version</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>need_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>need_adjustment</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>severity_weight</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>district_adjustment</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>capacity_weight</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>effective_from</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>approved_by</t>
         </is>
@@ -704,34 +712,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>dashboard_element</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>source_sheet</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>source_field(s)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>calculation_or_rule</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
@@ -858,170 +866,320 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>person_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>intake_date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>age</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>sex</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>district</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>village</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>language</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>contact_preference</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>consent_status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>last_reviewed</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>74</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Kota Setar</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Kampung Alor</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Alor Mengkudu</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Demo consent</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>P-0002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" t="n">
         <v>81</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Langkawi</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Kuah</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Family contact</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Demo consent</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>2026-11-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>67</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Jitra</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Demo consent</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>76</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Demo consent</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Baling</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Baling</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Family contact</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Demo consent</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
         </is>
       </c>
     </row>
@@ -1038,199 +1196,379 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>assessment_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>person_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>need_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>severity_1_5</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>urgency</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>frequency</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>evidence_note</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>assessed_by</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>assessed_at</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>A-0001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>transport</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Soon</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Hospital follow-up</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>AS-01</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>A-0002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>homecare</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Bathing and meal support</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>AS-01</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>A-0003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>P-0002</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>food</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Soon</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Irregular food access</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>AS-02</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2026-11-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P-0002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Soon</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Lives alone</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>AS-02</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>P-0003</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Wants social activities</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>AS-03</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>P-0004</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>homecare</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Needs help at home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>AS-04</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P-0005</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Income support enquiry</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>AS-05</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
         </is>
       </c>
     </row>
@@ -1247,10 +1585,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -1260,105 +1598,204 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>person_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>household_size</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>monthly_income_rm</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>carer_present</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>housing_type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>benefit_status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>eligibility_checked_at</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>1800</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Kampung house</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>P-0002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" t="n">
         <v>900</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Flat</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>2026-11-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Terrace house</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kampung house</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>800</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kampung house</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1387,122 +1824,392 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>district_code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>district_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>population_65_plus</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>service_density</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>data_confidence</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>last_refresh</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>KST</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Kota Setar</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>42000</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>LKW</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Langkawi</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" t="n">
         <v>12000</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>BLS</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Baling</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" t="n">
         <v>18000</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KPS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>26000</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KLM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SPT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PTP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Padang Terap</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PKS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pokok Sena</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PDG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pendang</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SIK</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sik</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>YAN</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Yan</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>11000</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BBH</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bandar Baharu</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>7000</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
@@ -1521,185 +2228,2050 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>provider_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>service_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>district</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>area_or_mukim</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>capacity_per_month</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>current_load</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>verified_at</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>contact_owner</t>
         </is>
       </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>phone_demo</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>opening_hours</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>assistance_offer</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>indicative_amount_rm</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>data_note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>PR-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Masjid Sharifah Fatimah</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Jitra</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Community coordinator</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>04-700 1001</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Visits, food and referral navigation</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>RM0 or donation</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PR-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Masjid Al-Bukhary Kedah</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Community coordinator</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>04-700 2002</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Community transport coordination</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>RM0 or donation</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PR-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Masjid Alor Merah</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Alor Merah</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Community coordinator</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>04-700 2003</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Food basket by assessment</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>RM0 or donation</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PR-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Masjid Taman Ria</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Community coordinator</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>04-700 3004</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Befriending and visits</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>RM0 or donation</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PR-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Masjid Bandar Baharu</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bandar Baharu</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Community coordinator</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>04-700 4005</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Referral to welfare support</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Subject to agency assessment</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PR-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kedah Islamic Welfare Association</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Case navigator</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>04-700 2006</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Case navigation and home visit</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Subject to eligibility</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PR-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WANIDA Kedah</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Case navigator</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>04-700 2007</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Volunteer matching</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Subject to screening</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PR-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PERKIM Kedah</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Case navigator</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>04-700 2008</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Welfare referral</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Subject to eligibility</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PR-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kedah Senior Citizens Network</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Demo coordinator</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>04-700 3009</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Peer support and activities</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PR-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MAIK / Baitulmal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Kaunter bantuan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>04-700 2010</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Zakat and welfare screening</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Amount depends on assessment</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PR-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LZNK</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Kaunter bantuan</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>04-700 2011</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Zakat application guidance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Amount depends on assessment</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PR-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JKM Kedah</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>welfare</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Kaunter bantuan</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>04-700 2012</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Assessment and referral</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Subject to eligibility</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PR-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PAWE Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Jitra</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>PAWE coordinator</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>04-700 1004</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Activities and peer support</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PR-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>PAWE Kota Setar</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>companionship</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Kota Setar</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Network lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>PR-002</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Hospital Langkawi</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>PAWE coordinator</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>04-700 2014</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Activities and peer support</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PR-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PAWE Kulim</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PAWE coordinator</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>04-700 4015</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Activities and peer support</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PR-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PAWE Sungai Petani</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PAWE coordinator</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>04-700 3016</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Activities and peer support</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Illustrative contact; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PR-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kedah Home Nursing 01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>homecare</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Service desk</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>04-700 2017</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Home nursing and wound care</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>RM80-RM180 per visit demo</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PR-018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Kedah Home Nursing 02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>homecare</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Service desk</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>04-700 3018</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Home care visits</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>RM60-RM150 per visit demo</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PR-019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Amanah Elderly Care Home 01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>residential</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Service desk</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>04-700 4019</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Short stay assessment</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>RM900-RM1800 monthly demo</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PR-020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Amanah Elderly Care Home 02</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>residential</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Service desk</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>04-700 2020</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Residential care enquiry</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>RM1000-RM2200 monthly demo</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PR-021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kedah Community Transport 01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>transport</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Jitra</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Transport desk</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>04-700 1021</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Appointment transport</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>RM0-RM40 trip demo</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PR-022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kedah Community Transport 02</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Transport desk</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>04-700 3022</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Appointment transport</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>RM0-RM40 trip demo</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PR-023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Meals-on-Wheels Kedah</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Service desk</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>04-700 2023</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Meal delivery</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>RM8-RM15 per meal demo</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PR-024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Neighbourhood Care Hub Kulim</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>homecare</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Kulim</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Service desk</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>04-700 4024</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Errands and home support</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>RM20-RM60 per visit demo</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PR-025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Volunteer Pool Jitra</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Kubang Pasu</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Jitra</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>04-700 1025</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Companion and escort</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PR-026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Volunteer Pool Alor Setar</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Kota Setar</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>04-700 2026</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Phone check-ins and errands</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PR-027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Volunteer Pool Sungai Petani</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sungai Petani</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>04-700 3027</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Transport coordination</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>RM0-RM20 donation demo</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PR-028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Volunteer Pool Baling</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Baling</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Baling</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>04-700 5028</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Food delivery and visits</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PR-029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Volunteer Pool Langkawi</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>Langkawi</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Hospital liaison</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>PR-003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Home Care Demo</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>homecare</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Kuah</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>04-700 6029</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Community visits</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>RM0 demo value</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PR-030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Kedah Silver Economy Coordination Desk</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>referral</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>Kota Setar</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Alor Setar</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Research team</t>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Coordination desk</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>04-700 2030</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-16:30</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Routes the case to the right desk</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>No direct payment; referral only</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Illustrative demo; verify before use</t>
         </is>
       </c>
     </row>
@@ -1716,154 +4288,223 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>referral_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>person_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>need_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>provider_id</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>referred_at</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>accepted_at</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>closed_at</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>outcome</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>wait_days</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>R-0001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>transport</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>PR-001</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PR-021</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Demo referral</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>R-0002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>homecare</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>PR-003</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PR-017</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Capacity check</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P-0002</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PR-028</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Langkawi route demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P-0003</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PR-013</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PAWE route demo</t>
         </is>
       </c>
     </row>
@@ -1880,94 +4521,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>outcome_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>referral_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>person_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>need_code</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>service_received</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>satisfaction_1_5</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>unmet_reason</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>recorded_at</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>O-0001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>R-0001</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>P-0001</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>transport</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Wait for confirmation</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>O-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>R-0004</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P-0003</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>companion</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pilot data</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
@@ -1989,41 +4666,41 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>label_en</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>label_bm</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>definition</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>